<commit_message>
docs(governance): add S26 governance closure report, required checks matrix, production gate, and update ledger
</commit_message>
<xml_diff>
--- a/التعلم/الاصلاح/Master_Remediation_Ledger_motion_محدث_S24_5.xlsx
+++ b/التعلم/الاصلاح/Master_Remediation_Ledger_motion_محدث_S24_5.xlsx
@@ -557,7 +557,7 @@
       </c>
       <c r="D5" s="28" t="inlineStr">
         <is>
-          <t>مكتمل ومثبت في S25</t>
+          <t>مكتمل ومثبت في S26</t>
         </is>
       </c>
       <c r="E5" s="28" t="inlineStr">
@@ -567,7 +567,7 @@
       </c>
       <c r="F5" s="28" t="inlineStr">
         <is>
-          <t>S25 مكتملة بالكامل</t>
+          <t>S26 مكتملة بالكامل (92/92 RESOLVED)</t>
         </is>
       </c>
       <c r="G5" s="28" t="inlineStr">
@@ -577,7 +577,7 @@
       </c>
       <c r="H5" s="28" t="inlineStr">
         <is>
-          <t>جاهز للمرحلة الختامية (S26 Governance)</t>
+          <t>جاهز لبدء مرحلة GUI / المنتج</t>
         </is>
       </c>
     </row>
@@ -8224,28 +8224,32 @@
       </c>
       <c r="L83" s="8" t="inlineStr">
         <is>
-          <t>بانتظار التحقق</t>
+          <t>تم التحقق بنجاح على main عبر Ruleset وBranch Protection ورفض مباشر</t>
         </is>
       </c>
       <c r="M83" s="8" t="inlineStr">
         <is>
-          <t>ENVIRONMENT_BLOCKED</t>
+          <t>RESOLVED</t>
         </is>
       </c>
       <c r="N83" s="8" t="inlineStr">
         <is>
-          <t>يُعيّن عند البدء</t>
-        </is>
-      </c>
-      <c r="O83" s="8" t="str"/>
+          <t>S26 Governance Engine</t>
+        </is>
+      </c>
+      <c r="O83" s="8" t="inlineStr">
+        <is>
+          <t>GOV-01 direct push rejected (GH013); GOV-02 force push rejected; GOV-03/04 blocked non-compliant PRs</t>
+        </is>
+      </c>
       <c r="P83" s="8" t="inlineStr">
         <is>
-          <t>Requires external GitHub repository settings / branch protection rules</t>
+          <t>GitHub Ruleset ID 24256136 + Classic Protection; PR #5 merged cleanly after 7/7 required checks green (Run 36739689585)</t>
         </is>
       </c>
       <c r="Q83" s="8" t="inlineStr">
         <is>
-          <t>S25 Re-Audit: External infrastructure prerequisite for production deployment</t>
+          <t>S26 Governance Closure: Ruleset + classic branch protection active and verified on main with zero bypass</t>
         </is>
       </c>
       <c r="R83" s="8" t="inlineStr">
@@ -8253,7 +8257,11 @@
           <t>البند 82؛ يتطلب صلاحية إدارة</t>
         </is>
       </c>
-      <c r="S83" s="8" t="str"/>
+      <c r="S83" s="8" t="inlineStr">
+        <is>
+          <t>PR #5 @ 69c1a5c</t>
+        </is>
+      </c>
     </row>
     <row r="84" ht="56" customHeight="1" s="12">
       <c r="A84" s="8" t="n">
@@ -10799,12 +10807,12 @@
       </c>
       <c r="C19" s="10" t="inlineStr">
         <is>
-          <t>ENVIRONMENT_BLOCKED</t>
+          <t>تم الإثبات بنجاح (RESOLVED)</t>
         </is>
       </c>
       <c r="D19" s="10" t="inlineStr">
         <is>
-          <t>يتطلب تفعيل branch protection ruleset من واجهة GitHub الإدارية</t>
+          <t>مُثبت في S26 عبر GitHub Ruleset ID 24256136 + Classic Protection، ورفض direct/force push (GH013)، و7/7 required checks إلزامية</t>
         </is>
       </c>
     </row>

</xml_diff>